<commit_message>
zakelijke staffel lezen aangepast
</commit_message>
<xml_diff>
--- a/Zakelijk/zakelijk_staffel.xlsx
+++ b/Zakelijk/zakelijk_staffel.xlsx
@@ -141,7 +141,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -163,11 +163,55 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -215,6 +259,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -610,7 +656,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Het systeem leest automatisch: Wassen Normaal, Intensief, Proteqt en Interieur Intensief, Interieur Proteqt.</t>
+          <t>Interieur: kolom F = bij Normaal/Intensief, kolom G = bij Proteqt. Was: kolom B=Normaal, C=Intensief, D=Proteqt.</t>
         </is>
       </c>
     </row>
@@ -654,14 +700,14 @@
       <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Interieur
-Intensief
+bij Normaal/Intensief
 (€/behandeling)</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Interieur
-Proteqt
+bij Proteqt
 (€/behandeling)</t>
         </is>
       </c>
@@ -1777,6 +1823,25 @@
           <t>Meer dan 50 wasbeurten per maand → Prijs op aanvraag via accountmanager</t>
         </is>
       </c>
+      <c r="B57" s="17" t="n"/>
+      <c r="C57" s="17" t="n"/>
+      <c r="D57" s="17" t="n"/>
+      <c r="E57" s="17" t="n"/>
+      <c r="F57" s="17" t="n"/>
+      <c r="G57" s="17" t="n"/>
+      <c r="H57" s="18" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Toelichting interieur-tarieven:</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Kolom F = interieur bij Normaal of Intensief wasprogramma (hoger tarief)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="13" t="inlineStr">
@@ -1786,7 +1851,7 @@
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>Gele cellen = Was-prijzen (aanpasbaar)</t>
+          <t>Kolom G = interieur bij Proteqt wasprogramma (lager tarief — loyaliteitskorting)</t>
         </is>
       </c>
       <c r="D59" s="15" t="inlineStr">

</xml_diff>